<commit_message>
Added evaluation tests to perform real model evaluations
</commit_message>
<xml_diff>
--- a/data/itau_cuenta_corriente_january_2026.xlsx
+++ b/data/itau_cuenta_corriente_january_2026.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Cuenta Corriente" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cuenta Corriente" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -469,7 +469,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F36"/>
+  <dimension ref="A1:F63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1411,13 +1411,823 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="9" t="inlineStr">
+      <c r="A36" s="6" t="inlineStr">
+        <is>
+          <t>2026-01-04</t>
+        </is>
+      </c>
+      <c r="B36" s="6" t="inlineStr">
+        <is>
+          <t>RESTAURANT LA PARRILLA</t>
+        </is>
+      </c>
+      <c r="C36" s="7" t="n">
+        <v>-18500</v>
+      </c>
+      <c r="D36" s="6" t="inlineStr">
+        <is>
+          <t>UYU</t>
+        </is>
+      </c>
+      <c r="E36" s="6" t="inlineStr">
+        <is>
+          <t>Itaú Cuenta Corriente ****4821</t>
+        </is>
+      </c>
+      <c r="F36" s="6" t="inlineStr">
+        <is>
+          <t>REF1029</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>2026-01-04</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>EVAL DINE BASELINE 1</t>
+        </is>
+      </c>
+      <c r="C37" s="5" t="n">
+        <v>-1500</v>
+      </c>
+      <c r="D37" s="4" t="inlineStr">
+        <is>
+          <t>UYU</t>
+        </is>
+      </c>
+      <c r="E37" s="4" t="inlineStr">
+        <is>
+          <t>Itaú Cuenta Corriente ****4821</t>
+        </is>
+      </c>
+      <c r="F37" s="4" t="inlineStr">
+        <is>
+          <t>REF1030</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="6" t="inlineStr">
+        <is>
+          <t>2026-01-04</t>
+        </is>
+      </c>
+      <c r="B38" s="6" t="inlineStr">
+        <is>
+          <t>EVAL DINE BASELINE 2</t>
+        </is>
+      </c>
+      <c r="C38" s="7" t="n">
+        <v>-1600</v>
+      </c>
+      <c r="D38" s="6" t="inlineStr">
+        <is>
+          <t>UYU</t>
+        </is>
+      </c>
+      <c r="E38" s="6" t="inlineStr">
+        <is>
+          <t>Itaú Cuenta Corriente ****4821</t>
+        </is>
+      </c>
+      <c r="F38" s="6" t="inlineStr">
+        <is>
+          <t>REF1031</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>2026-01-18</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>TRANSFERENCIA EVAL ROUND</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="n">
+        <v>-50000</v>
+      </c>
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t>UYU</t>
+        </is>
+      </c>
+      <c r="E39" s="4" t="inlineStr">
+        <is>
+          <t>Itaú Cuenta Corriente ****4821</t>
+        </is>
+      </c>
+      <c r="F39" s="4" t="inlineStr">
+        <is>
+          <t>REF1032</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="6" t="inlineStr">
+        <is>
+          <t>2026-01-20</t>
+        </is>
+      </c>
+      <c r="B40" s="6" t="inlineStr">
+        <is>
+          <t>TIENDA XYZ EVAL RAPID</t>
+        </is>
+      </c>
+      <c r="C40" s="7" t="n">
+        <v>-800</v>
+      </c>
+      <c r="D40" s="6" t="inlineStr">
+        <is>
+          <t>UYU</t>
+        </is>
+      </c>
+      <c r="E40" s="6" t="inlineStr">
+        <is>
+          <t>Itaú Cuenta Corriente ****4821</t>
+        </is>
+      </c>
+      <c r="F40" s="6" t="inlineStr">
+        <is>
+          <t>REF1033</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>2026-01-20</t>
+        </is>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>TIENDA XYZ EVAL RAPID</t>
+        </is>
+      </c>
+      <c r="C41" s="5" t="n">
+        <v>-800</v>
+      </c>
+      <c r="D41" s="4" t="inlineStr">
+        <is>
+          <t>UYU</t>
+        </is>
+      </c>
+      <c r="E41" s="4" t="inlineStr">
+        <is>
+          <t>Itaú Cuenta Corriente ****4821</t>
+        </is>
+      </c>
+      <c r="F41" s="4" t="inlineStr">
+        <is>
+          <t>REF1034</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="6" t="inlineStr">
+        <is>
+          <t>2026-01-20</t>
+        </is>
+      </c>
+      <c r="B42" s="6" t="inlineStr">
+        <is>
+          <t>TIENDA XYZ EVAL RAPID</t>
+        </is>
+      </c>
+      <c r="C42" s="7" t="n">
+        <v>-800</v>
+      </c>
+      <c r="D42" s="6" t="inlineStr">
+        <is>
+          <t>UYU</t>
+        </is>
+      </c>
+      <c r="E42" s="6" t="inlineStr">
+        <is>
+          <t>Itaú Cuenta Corriente ****4821</t>
+        </is>
+      </c>
+      <c r="F42" s="6" t="inlineStr">
+        <is>
+          <t>REF1035</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>2026-01-20</t>
+        </is>
+      </c>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>TIENDA XYZ EVAL RAPID</t>
+        </is>
+      </c>
+      <c r="C43" s="5" t="n">
+        <v>-800</v>
+      </c>
+      <c r="D43" s="4" t="inlineStr">
+        <is>
+          <t>UYU</t>
+        </is>
+      </c>
+      <c r="E43" s="4" t="inlineStr">
+        <is>
+          <t>Itaú Cuenta Corriente ****4821</t>
+        </is>
+      </c>
+      <c r="F43" s="4" t="inlineStr">
+        <is>
+          <t>REF1036</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="6" t="inlineStr">
+        <is>
+          <t>2026-01-20</t>
+        </is>
+      </c>
+      <c r="B44" s="6" t="inlineStr">
+        <is>
+          <t>TIENDA XYZ EVAL RAPID</t>
+        </is>
+      </c>
+      <c r="C44" s="7" t="n">
+        <v>-800</v>
+      </c>
+      <c r="D44" s="6" t="inlineStr">
+        <is>
+          <t>UYU</t>
+        </is>
+      </c>
+      <c r="E44" s="6" t="inlineStr">
+        <is>
+          <t>Itaú Cuenta Corriente ****4821</t>
+        </is>
+      </c>
+      <c r="F44" s="6" t="inlineStr">
+        <is>
+          <t>REF1037</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>2026-01-11</t>
+        </is>
+      </c>
+      <c r="B45" s="4" t="inlineStr">
+        <is>
+          <t>EVAL ALIAS NETFLIX</t>
+        </is>
+      </c>
+      <c r="C45" s="5" t="n">
+        <v>-720</v>
+      </c>
+      <c r="D45" s="4" t="inlineStr">
+        <is>
+          <t>UYU</t>
+        </is>
+      </c>
+      <c r="E45" s="4" t="inlineStr">
+        <is>
+          <t>Itaú Cuenta Corriente ****4821</t>
+        </is>
+      </c>
+      <c r="F45" s="4" t="inlineStr">
+        <is>
+          <t>REF1038</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="6" t="inlineStr">
+        <is>
+          <t>2026-01-12</t>
+        </is>
+      </c>
+      <c r="B46" s="6" t="inlineStr">
+        <is>
+          <t>EVAL UBER EATS STAR</t>
+        </is>
+      </c>
+      <c r="C46" s="7" t="n">
+        <v>-450</v>
+      </c>
+      <c r="D46" s="6" t="inlineStr">
+        <is>
+          <t>UYU</t>
+        </is>
+      </c>
+      <c r="E46" s="6" t="inlineStr">
+        <is>
+          <t>Itaú Cuenta Corriente ****4821</t>
+        </is>
+      </c>
+      <c r="F46" s="6" t="inlineStr">
+        <is>
+          <t>REF1039</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
+      <c r="B47" s="4" t="inlineStr">
+        <is>
+          <t>EVAL MERCADOLIBRE</t>
+        </is>
+      </c>
+      <c r="C47" s="5" t="n">
+        <v>-800</v>
+      </c>
+      <c r="D47" s="4" t="inlineStr">
+        <is>
+          <t>UYU</t>
+        </is>
+      </c>
+      <c r="E47" s="4" t="inlineStr">
+        <is>
+          <t>Itaú Cuenta Corriente ****4821</t>
+        </is>
+      </c>
+      <c r="F47" s="4" t="inlineStr">
+        <is>
+          <t>REF1040</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="6" t="inlineStr">
+        <is>
+          <t>2026-01-14</t>
+        </is>
+      </c>
+      <c r="B48" s="6" t="inlineStr">
+        <is>
+          <t>EVAL BAIT SHOP 00</t>
+        </is>
+      </c>
+      <c r="C48" s="7" t="n">
+        <v>-248</v>
+      </c>
+      <c r="D48" s="6" t="inlineStr">
+        <is>
+          <t>UYU</t>
+        </is>
+      </c>
+      <c r="E48" s="6" t="inlineStr">
+        <is>
+          <t>Itaú Cuenta Corriente ****4821</t>
+        </is>
+      </c>
+      <c r="F48" s="6" t="inlineStr">
+        <is>
+          <t>REF1041</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>2026-01-15</t>
+        </is>
+      </c>
+      <c r="B49" s="4" t="inlineStr">
+        <is>
+          <t>EVAL BAIT SHOP 01</t>
+        </is>
+      </c>
+      <c r="C49" s="5" t="n">
+        <v>-251</v>
+      </c>
+      <c r="D49" s="4" t="inlineStr">
+        <is>
+          <t>UYU</t>
+        </is>
+      </c>
+      <c r="E49" s="4" t="inlineStr">
+        <is>
+          <t>Itaú Cuenta Corriente ****4821</t>
+        </is>
+      </c>
+      <c r="F49" s="4" t="inlineStr">
+        <is>
+          <t>REF1042</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="6" t="inlineStr">
+        <is>
+          <t>2026-01-16</t>
+        </is>
+      </c>
+      <c r="B50" s="6" t="inlineStr">
+        <is>
+          <t>EVAL BAIT SHOP 02</t>
+        </is>
+      </c>
+      <c r="C50" s="7" t="n">
+        <v>-254</v>
+      </c>
+      <c r="D50" s="6" t="inlineStr">
+        <is>
+          <t>UYU</t>
+        </is>
+      </c>
+      <c r="E50" s="6" t="inlineStr">
+        <is>
+          <t>Itaú Cuenta Corriente ****4821</t>
+        </is>
+      </c>
+      <c r="F50" s="6" t="inlineStr">
+        <is>
+          <t>REF1043</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>2026-01-17</t>
+        </is>
+      </c>
+      <c r="B51" s="4" t="inlineStr">
+        <is>
+          <t>EVAL BAIT SHOP 03</t>
+        </is>
+      </c>
+      <c r="C51" s="5" t="n">
+        <v>-257</v>
+      </c>
+      <c r="D51" s="4" t="inlineStr">
+        <is>
+          <t>UYU</t>
+        </is>
+      </c>
+      <c r="E51" s="4" t="inlineStr">
+        <is>
+          <t>Itaú Cuenta Corriente ****4821</t>
+        </is>
+      </c>
+      <c r="F51" s="4" t="inlineStr">
+        <is>
+          <t>REF1044</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="6" t="inlineStr">
+        <is>
+          <t>2026-01-18</t>
+        </is>
+      </c>
+      <c r="B52" s="6" t="inlineStr">
+        <is>
+          <t>EVAL BAIT SHOP 04</t>
+        </is>
+      </c>
+      <c r="C52" s="7" t="n">
+        <v>-260</v>
+      </c>
+      <c r="D52" s="6" t="inlineStr">
+        <is>
+          <t>UYU</t>
+        </is>
+      </c>
+      <c r="E52" s="6" t="inlineStr">
+        <is>
+          <t>Itaú Cuenta Corriente ****4821</t>
+        </is>
+      </c>
+      <c r="F52" s="6" t="inlineStr">
+        <is>
+          <t>REF1045</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>2026-01-19</t>
+        </is>
+      </c>
+      <c r="B53" s="4" t="inlineStr">
+        <is>
+          <t>EVAL BAIT SHOP 05</t>
+        </is>
+      </c>
+      <c r="C53" s="5" t="n">
+        <v>-263</v>
+      </c>
+      <c r="D53" s="4" t="inlineStr">
+        <is>
+          <t>UYU</t>
+        </is>
+      </c>
+      <c r="E53" s="4" t="inlineStr">
+        <is>
+          <t>Itaú Cuenta Corriente ****4821</t>
+        </is>
+      </c>
+      <c r="F53" s="4" t="inlineStr">
+        <is>
+          <t>REF1046</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="6" t="inlineStr">
+        <is>
+          <t>2026-01-20</t>
+        </is>
+      </c>
+      <c r="B54" s="6" t="inlineStr">
+        <is>
+          <t>EVAL BAIT SHOP 06</t>
+        </is>
+      </c>
+      <c r="C54" s="7" t="n">
+        <v>-266</v>
+      </c>
+      <c r="D54" s="6" t="inlineStr">
+        <is>
+          <t>UYU</t>
+        </is>
+      </c>
+      <c r="E54" s="6" t="inlineStr">
+        <is>
+          <t>Itaú Cuenta Corriente ****4821</t>
+        </is>
+      </c>
+      <c r="F54" s="6" t="inlineStr">
+        <is>
+          <t>REF1047</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>2026-01-21</t>
+        </is>
+      </c>
+      <c r="B55" s="4" t="inlineStr">
+        <is>
+          <t>EVAL BAIT SHOP 07</t>
+        </is>
+      </c>
+      <c r="C55" s="5" t="n">
+        <v>-269</v>
+      </c>
+      <c r="D55" s="4" t="inlineStr">
+        <is>
+          <t>UYU</t>
+        </is>
+      </c>
+      <c r="E55" s="4" t="inlineStr">
+        <is>
+          <t>Itaú Cuenta Corriente ****4821</t>
+        </is>
+      </c>
+      <c r="F55" s="4" t="inlineStr">
+        <is>
+          <t>REF1048</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="6" t="inlineStr">
+        <is>
+          <t>2026-01-22</t>
+        </is>
+      </c>
+      <c r="B56" s="6" t="inlineStr">
+        <is>
+          <t>EVAL BAIT SHOP 08</t>
+        </is>
+      </c>
+      <c r="C56" s="7" t="n">
+        <v>-272</v>
+      </c>
+      <c r="D56" s="6" t="inlineStr">
+        <is>
+          <t>UYU</t>
+        </is>
+      </c>
+      <c r="E56" s="6" t="inlineStr">
+        <is>
+          <t>Itaú Cuenta Corriente ****4821</t>
+        </is>
+      </c>
+      <c r="F56" s="6" t="inlineStr">
+        <is>
+          <t>REF1049</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>2026-01-23</t>
+        </is>
+      </c>
+      <c r="B57" s="4" t="inlineStr">
+        <is>
+          <t>EVAL BAIT SHOP 09</t>
+        </is>
+      </c>
+      <c r="C57" s="5" t="n">
+        <v>-275</v>
+      </c>
+      <c r="D57" s="4" t="inlineStr">
+        <is>
+          <t>UYU</t>
+        </is>
+      </c>
+      <c r="E57" s="4" t="inlineStr">
+        <is>
+          <t>Itaú Cuenta Corriente ****4821</t>
+        </is>
+      </c>
+      <c r="F57" s="4" t="inlineStr">
+        <is>
+          <t>REF1050</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="6" t="inlineStr">
+        <is>
+          <t>2026-01-24</t>
+        </is>
+      </c>
+      <c r="B58" s="6" t="inlineStr">
+        <is>
+          <t>EVAL BAIT SHOP 10</t>
+        </is>
+      </c>
+      <c r="C58" s="7" t="n">
+        <v>-278</v>
+      </c>
+      <c r="D58" s="6" t="inlineStr">
+        <is>
+          <t>UYU</t>
+        </is>
+      </c>
+      <c r="E58" s="6" t="inlineStr">
+        <is>
+          <t>Itaú Cuenta Corriente ****4821</t>
+        </is>
+      </c>
+      <c r="F58" s="6" t="inlineStr">
+        <is>
+          <t>REF1051</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="4" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
+        </is>
+      </c>
+      <c r="B59" s="4" t="inlineStr">
+        <is>
+          <t>EVAL BAIT SHOP 11</t>
+        </is>
+      </c>
+      <c r="C59" s="5" t="n">
+        <v>-281</v>
+      </c>
+      <c r="D59" s="4" t="inlineStr">
+        <is>
+          <t>UYU</t>
+        </is>
+      </c>
+      <c r="E59" s="4" t="inlineStr">
+        <is>
+          <t>Itaú Cuenta Corriente ****4821</t>
+        </is>
+      </c>
+      <c r="F59" s="4" t="inlineStr">
+        <is>
+          <t>REF1052</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="6" t="inlineStr">
+        <is>
+          <t>2026-01-26</t>
+        </is>
+      </c>
+      <c r="B60" s="6" t="inlineStr">
+        <is>
+          <t>EVAL BAIT SHOP 12</t>
+        </is>
+      </c>
+      <c r="C60" s="7" t="n">
+        <v>-284</v>
+      </c>
+      <c r="D60" s="6" t="inlineStr">
+        <is>
+          <t>UYU</t>
+        </is>
+      </c>
+      <c r="E60" s="6" t="inlineStr">
+        <is>
+          <t>Itaú Cuenta Corriente ****4821</t>
+        </is>
+      </c>
+      <c r="F60" s="6" t="inlineStr">
+        <is>
+          <t>REF1053</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="4" t="inlineStr">
+        <is>
+          <t>2026-01-27</t>
+        </is>
+      </c>
+      <c r="B61" s="4" t="inlineStr">
+        <is>
+          <t>EVAL BAIT SHOP 13</t>
+        </is>
+      </c>
+      <c r="C61" s="5" t="n">
+        <v>-287</v>
+      </c>
+      <c r="D61" s="4" t="inlineStr">
+        <is>
+          <t>UYU</t>
+        </is>
+      </c>
+      <c r="E61" s="4" t="inlineStr">
+        <is>
+          <t>Itaú Cuenta Corriente ****4821</t>
+        </is>
+      </c>
+      <c r="F61" s="4" t="inlineStr">
+        <is>
+          <t>REF1054</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="6" t="inlineStr">
+        <is>
+          <t>2026-01-28</t>
+        </is>
+      </c>
+      <c r="B62" s="6" t="inlineStr">
+        <is>
+          <t>EVAL BAIT SHOP 14</t>
+        </is>
+      </c>
+      <c r="C62" s="7" t="n">
+        <v>-290</v>
+      </c>
+      <c r="D62" s="6" t="inlineStr">
+        <is>
+          <t>UYU</t>
+        </is>
+      </c>
+      <c r="E62" s="6" t="inlineStr">
+        <is>
+          <t>Itaú Cuenta Corriente ****4821</t>
+        </is>
+      </c>
+      <c r="F62" s="6" t="inlineStr">
+        <is>
+          <t>REF1055</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="9" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C36" s="10">
-        <f>SUM(C7:C35)</f>
+      <c r="C63" s="10">
+        <f>SUM(C7:C62)</f>
         <v/>
       </c>
     </row>

</xml_diff>